<commit_message>
Exclude COO from personnel contract workbook
</commit_message>
<xml_diff>
--- a/projects/PetroUrdaneta-FDP9/compensation/personnel_base_salary_contract_types.xlsx
+++ b/projects/PetroUrdaneta-FDP9/compensation/personnel_base_salary_contract_types.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Contract Rules'!$B$2:$M$23</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Personnel!$B$2:$Y$29</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Personnel!$B$2:$Y$28</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -294,15 +294,15 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="C17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: row number.</t>
+    <comment ref="D9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Position.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -327,7 +327,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D9" authorId="0">
+    <comment ref="D10" authorId="0">
       <text>
         <r>
           <rPr>
@@ -360,7 +360,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D10" authorId="0">
+    <comment ref="D11" authorId="0">
       <text>
         <r>
           <rPr>
@@ -393,7 +393,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D11" authorId="0">
+    <comment ref="D12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -426,7 +426,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D12" authorId="0">
+    <comment ref="D13" authorId="0">
       <text>
         <r>
           <rPr>
@@ -459,7 +459,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D13" authorId="0">
+    <comment ref="D14" authorId="0">
       <text>
         <r>
           <rPr>
@@ -492,7 +492,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D14" authorId="0">
+    <comment ref="D15" authorId="0">
       <text>
         <r>
           <rPr>
@@ -525,7 +525,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D15" authorId="0">
+    <comment ref="D16" authorId="0">
       <text>
         <r>
           <rPr>
@@ -558,15 +558,15 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Position.</t>
+    <comment ref="E9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Person.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -591,15 +591,15 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Position.</t>
+    <comment ref="E10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Person.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -624,7 +624,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E9" authorId="0">
+    <comment ref="E11" authorId="0">
       <text>
         <r>
           <rPr>
@@ -657,7 +657,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E10" authorId="0">
+    <comment ref="E12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -690,7 +690,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E11" authorId="0">
+    <comment ref="E13" authorId="0">
       <text>
         <r>
           <rPr>
@@ -723,7 +723,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E12" authorId="0">
+    <comment ref="E14" authorId="0">
       <text>
         <r>
           <rPr>
@@ -756,7 +756,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E13" authorId="0">
+    <comment ref="E15" authorId="0">
       <text>
         <r>
           <rPr>
@@ -789,7 +789,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E14" authorId="0">
+    <comment ref="E16" authorId="0">
       <text>
         <r>
           <rPr>
@@ -822,15 +822,1335 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E15" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Person.</t>
+    <comment ref="F9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>8</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="K9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="K10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="K11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="K12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="K13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="K14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="K15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="K16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; initially appointed General Manager of PU on secondment; transitions to Local — Venezuela from M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Expat; initially appointed Technical Manager of PU on secondment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Remote role. Local / Fixed is an editable assumption pending confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Rotation confirmed from prior instructions; Expat contract is an editable assumption.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Local in Maracaibo or staff house; no cash housing allowance by default.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Local in Maracaibo or staff house; no cash housing allowance by default.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="Y9" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Base Salary (Annual).</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -855,15 +2175,15 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Person.</t>
+    <comment ref="Y10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Base Salary (Annual).</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -888,15 +2208,15 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="E17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Person.</t>
+    <comment ref="Y11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Base Salary (Annual).</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -921,1492 +2241,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F9" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F10" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F11" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F12" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F14" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F15" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H9" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H10" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H11" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H12" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H14" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H15" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="H17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Work arrangement must be Fixed or Rotation. Remote is documented in Notes, not treated as a fourth contract type.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J9" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J10" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J11" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J12" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J14" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J15" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="J17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K9" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K10" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K11" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K12" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K14" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K15" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="K17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Confirmed means directly established in prior instructions; Assumption remains editable and requires confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L9" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Expat classification carried forward from prior instructions.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>1</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L10" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>16</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L11" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; initially appointed General Manager of PU on secondment; transitions to Local — Venezuela from M7.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L12" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>16</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Expat; initially appointed Technical Manager of PU on secondment.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>1</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L14" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Remote role. Local / Fixed is an editable assumption pending confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>1</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L15" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Rotation confirmed from prior instructions; Expat contract is an editable assumption.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>16</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Local in Maracaibo or staff house; no cash housing allowance by default.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>16</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="L17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Local in Maracaibo or staff house; no cash housing allowance by default.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>16</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="Y9" authorId="0">
+    <comment ref="Y12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -2439,7 +2274,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="Y10" authorId="0">
+    <comment ref="Y13" authorId="0">
       <text>
         <r>
           <rPr>
@@ -2472,7 +2307,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="Y11" authorId="0">
+    <comment ref="Y14" authorId="0">
       <text>
         <r>
           <rPr>
@@ -2505,7 +2340,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="Y12" authorId="0">
+    <comment ref="Y15" authorId="0">
       <text>
         <r>
           <rPr>
@@ -2538,139 +2373,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="Y13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Base Salary (Annual).</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>4</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="Y14" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Base Salary (Annual).</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>4</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="Y15" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Base Salary (Annual).</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>4</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
     <comment ref="Y16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Base Salary (Annual).</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>4</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="Y17" authorId="0">
       <text>
         <r>
           <rPr>
@@ -4137,15 +3840,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="116">
   <si>
     <t xml:space="preserve">Personnel — Monthly Base Salary and Contract Classification</t>
   </si>
   <si>
-    <t xml:space="preserve">Repatriates transition to Local — Venezuela from M7 after a one-time transition bonus | Fixed and Rotation shown separately</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD | M1–M12 = annual base salary / 12 | One-time transition bonus is not included in monthly base salary</t>
+    <t xml:space="preserve">COO / PU General Manager excluded and treated separately | Repatriates transition to Local — Venezuela from M7 after a one-time transition bonus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD | M1–M12 = annual base salary / 12 | One-time transition bonus is not included in monthly base salary | 8 people only</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -4217,63 +3920,54 @@
     <t xml:space="preserve">Base Salary Annual</t>
   </si>
   <si>
-    <t xml:space="preserve">COO / PU General Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Martin del Castillo</t>
+    <t xml:space="preserve">EPCM &amp; Engineering Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juan Conde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repatriate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eligible — one-time; amount TBD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drilling &amp; Well Services Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alexander Stulme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repatriate; initially appointed General Manager of PU on secondment; transitions to Local — Venezuela from M7.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operations &amp; Maintenance Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Félix Valderrama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical Manager (Geosciences)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alan McKeon</t>
   </si>
   <si>
     <t xml:space="preserve">Expat</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixed</t>
-  </si>
-  <si>
     <t xml:space="preserve">Not applicable</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expat classification carried forward from prior instructions.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EPCM &amp; Engineering Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juan Conde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repatriate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eligible — one-time; amount TBD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drilling &amp; Well Services Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alexander Stulme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repatriate; initially appointed General Manager of PU on secondment; transitions to Local — Venezuela from M7.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operations &amp; Maintenance Manager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Félix Valderrama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Technical Manager (Geosciences)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alan McKeon</t>
-  </si>
-  <si>
     <t xml:space="preserve">Expat; initially appointed Technical Manager of PU on secondment.</t>
   </si>
   <si>
@@ -4319,7 +4013,7 @@
     <t xml:space="preserve">Leticia Almeida</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL — 9 PEOPLE</t>
+    <t xml:space="preserve">TOTAL — 8 PEOPLE (COO EXCLUDED)</t>
   </si>
   <si>
     <t xml:space="preserve">CLASSIFICATION SUMMARY</t>
@@ -5069,11 +4763,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="C3:Y29"/>
+  <dimension ref="C3:Y28"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
@@ -5252,14 +4946,14 @@
       </c>
       <c r="G9" s="11" t="str">
         <f aca="false">IF(F9="Expat","Yes","No")</f>
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I9" s="12" t="str">
         <f aca="false">IF(F9="Repatriate","Local — Venezuela",F9)</f>
-        <v>Expat</v>
+        <v>Local — Venezuela</v>
       </c>
       <c r="J9" s="13" t="s">
         <v>30</v>
@@ -5272,54 +4966,54 @@
       </c>
       <c r="M9" s="14" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="N9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="O9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="P9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="Q9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="R9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="S9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="T9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="U9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="V9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="W9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="X9" s="15" t="n">
         <f aca="false">$Y9/12</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
       <c r="Y9" s="16" t="n">
-        <v>360000</v>
+        <v>216000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5333,7 +5027,7 @@
         <v>34</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G10" s="11" t="str">
         <f aca="false">IF(F10="Expat","Yes","No")</f>
@@ -5347,64 +5041,64 @@
         <v>Local — Venezuela</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>31</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="N10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="O10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="P10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="Q10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="R10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="S10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="T10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="U10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="V10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="W10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="X10" s="15" t="n">
         <f aca="false">$Y10/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="Y10" s="17" t="n">
-        <v>216000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5412,13 +5106,13 @@
         <v>3</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G11" s="11" t="str">
         <f aca="false">IF(F11="Expat","Yes","No")</f>
@@ -5432,64 +5126,64 @@
         <v>Local — Venezuela</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="K11" s="10" t="s">
         <v>31</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="M11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="N11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="O11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="P11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="Q11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="R11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="S11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="T11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="U11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="V11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="W11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="X11" s="15" t="n">
         <f aca="false">$Y11/12</f>
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="Y11" s="17" t="n">
-        <v>180000</v>
+        <v>216000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5497,84 +5191,84 @@
         <v>4</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G12" s="11" t="str">
         <f aca="false">IF(F12="Expat","Yes","No")</f>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I12" s="12" t="str">
         <f aca="false">IF(F12="Repatriate","Local — Venezuela",F12)</f>
-        <v>Local — Venezuela</v>
+        <v>Expat</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>31</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="M12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="N12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="O12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="P12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="Q12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="R12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="S12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="T12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="U12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="V12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="W12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="X12" s="15" t="n">
         <f aca="false">$Y12/12</f>
-        <v>18000</v>
+        <v>15000</v>
       </c>
       <c r="Y12" s="17" t="n">
-        <v>216000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5588,78 +5282,78 @@
         <v>44</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G13" s="11" t="str">
         <f aca="false">IF(F13="Expat","Yes","No")</f>
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I13" s="12" t="str">
         <f aca="false">IF(F13="Repatriate","Local — Venezuela",F13)</f>
-        <v>Expat</v>
+        <v>Local</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="L13" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="M13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="N13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="O13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="P13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="Q13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="R13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="S13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="T13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="U13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="V13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="W13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="X13" s="15" t="n">
         <f aca="false">$Y13/12</f>
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="Y13" s="17" t="n">
-        <v>180000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5667,84 +5361,84 @@
         <v>6</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="G14" s="11" t="str">
         <f aca="false">IF(F14="Expat","Yes","No")</f>
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="I14" s="12" t="str">
         <f aca="false">IF(F14="Repatriate","Local — Venezuela",F14)</f>
-        <v>Local</v>
+        <v>Expat</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="L14" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="N14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="O14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="P14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="Q14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="R14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="S14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="T14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="U14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="V14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="W14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="X14" s="15" t="n">
         <f aca="false">$Y14/12</f>
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="Y14" s="17" t="n">
-        <v>120000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5752,84 +5446,84 @@
         <v>7</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G15" s="11" t="str">
         <f aca="false">IF(F15="Expat","Yes","No")</f>
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="I15" s="12" t="str">
         <f aca="false">IF(F15="Repatriate","Local — Venezuela",F15)</f>
-        <v>Expat</v>
+        <v>Local</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="L15" s="8" t="s">
         <v>54</v>
       </c>
       <c r="M15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="N15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="O15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="P15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="Q15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="R15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="S15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="T15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="U15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="V15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="W15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="X15" s="15" t="n">
         <f aca="false">$Y15/12</f>
-        <v>15000</v>
+        <v>4000</v>
       </c>
       <c r="Y15" s="17" t="n">
-        <v>180000</v>
+        <v>48000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5843,7 +5537,7 @@
         <v>56</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G16" s="11" t="str">
         <f aca="false">IF(F16="Expat","Yes","No")</f>
@@ -5857,13 +5551,13 @@
         <v>Local</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="K16" s="10" t="s">
         <v>31</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="M16" s="15" t="n">
         <f aca="false">$Y16/12</f>
@@ -5917,193 +5611,120 @@
         <v>48000</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D17" s="8" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C17" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="18"/>
+      <c r="M17" s="19" t="n">
+        <f aca="false">SUM(M9:M16)</f>
+        <v>99000</v>
+      </c>
+      <c r="N17" s="20" t="n">
+        <f aca="false">SUM(N9:N16)</f>
+        <v>99000</v>
+      </c>
+      <c r="O17" s="20" t="n">
+        <f aca="false">SUM(O9:O16)</f>
+        <v>99000</v>
+      </c>
+      <c r="P17" s="20" t="n">
+        <f aca="false">SUM(P9:P16)</f>
+        <v>99000</v>
+      </c>
+      <c r="Q17" s="20" t="n">
+        <f aca="false">SUM(Q9:Q16)</f>
+        <v>99000</v>
+      </c>
+      <c r="R17" s="20" t="n">
+        <f aca="false">SUM(R9:R16)</f>
+        <v>99000</v>
+      </c>
+      <c r="S17" s="20" t="n">
+        <f aca="false">SUM(S9:S16)</f>
+        <v>99000</v>
+      </c>
+      <c r="T17" s="20" t="n">
+        <f aca="false">SUM(T9:T16)</f>
+        <v>99000</v>
+      </c>
+      <c r="U17" s="20" t="n">
+        <f aca="false">SUM(U9:U16)</f>
+        <v>99000</v>
+      </c>
+      <c r="V17" s="20" t="n">
+        <f aca="false">SUM(V9:V16)</f>
+        <v>99000</v>
+      </c>
+      <c r="W17" s="20" t="n">
+        <f aca="false">SUM(W9:W16)</f>
+        <v>99000</v>
+      </c>
+      <c r="X17" s="20" t="n">
+        <f aca="false">SUM(X9:X16)</f>
+        <v>99000</v>
+      </c>
+      <c r="Y17" s="19" t="n">
+        <f aca="false">SUM(Y9:Y16)</f>
+        <v>1188000</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C20" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="21"/>
+      <c r="P20" s="21"/>
+      <c r="Q20" s="21"/>
+      <c r="R20" s="21"/>
+      <c r="S20" s="21"/>
+      <c r="T20" s="21"/>
+      <c r="U20" s="21"/>
+      <c r="V20" s="21"/>
+      <c r="W20" s="21"/>
+      <c r="X20" s="21"/>
+      <c r="Y20" s="21"/>
+    </row>
+    <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C21" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="G17" s="11" t="str">
-        <f aca="false">IF(F17="Expat","Yes","No")</f>
-        <v>No</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="I17" s="12" t="str">
-        <f aca="false">IF(F17="Repatriate","Local — Venezuela",F17)</f>
-        <v>Local</v>
-      </c>
-      <c r="J17" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="K17" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="L17" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="M17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="N17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="O17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="P17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="Q17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="R17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="S17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="T17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="U17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="V17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="W17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="X17" s="15" t="n">
-        <f aca="false">$Y17/12</f>
-        <v>4000</v>
-      </c>
-      <c r="Y17" s="17" t="n">
-        <v>48000</v>
+      <c r="D21" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>61</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="19" t="n">
-        <f aca="false">SUM(M9:M17)</f>
-        <v>129000</v>
-      </c>
-      <c r="N18" s="20" t="n">
-        <f aca="false">SUM(N9:N17)</f>
-        <v>129000</v>
-      </c>
-      <c r="O18" s="20" t="n">
-        <f aca="false">SUM(O9:O17)</f>
-        <v>129000</v>
-      </c>
-      <c r="P18" s="20" t="n">
-        <f aca="false">SUM(P9:P17)</f>
-        <v>129000</v>
-      </c>
-      <c r="Q18" s="20" t="n">
-        <f aca="false">SUM(Q9:Q17)</f>
-        <v>129000</v>
-      </c>
-      <c r="R18" s="20" t="n">
-        <f aca="false">SUM(R9:R17)</f>
-        <v>129000</v>
-      </c>
-      <c r="S18" s="20" t="n">
-        <f aca="false">SUM(S9:S17)</f>
-        <v>129000</v>
-      </c>
-      <c r="T18" s="20" t="n">
-        <f aca="false">SUM(T9:T17)</f>
-        <v>129000</v>
-      </c>
-      <c r="U18" s="20" t="n">
-        <f aca="false">SUM(U9:U17)</f>
-        <v>129000</v>
-      </c>
-      <c r="V18" s="20" t="n">
-        <f aca="false">SUM(V9:V17)</f>
-        <v>129000</v>
-      </c>
-      <c r="W18" s="20" t="n">
-        <f aca="false">SUM(W9:W17)</f>
-        <v>129000</v>
-      </c>
-      <c r="X18" s="20" t="n">
-        <f aca="false">SUM(X9:X17)</f>
-        <v>129000</v>
-      </c>
-      <c r="Y18" s="19" t="n">
-        <f aca="false">SUM(Y9:Y17)</f>
-        <v>1548000</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-      <c r="N21" s="21"/>
-      <c r="O21" s="21"/>
-      <c r="P21" s="21"/>
-      <c r="Q21" s="21"/>
-      <c r="R21" s="21"/>
-      <c r="S21" s="21"/>
-      <c r="T21" s="21"/>
-      <c r="U21" s="21"/>
-      <c r="V21" s="21"/>
-      <c r="W21" s="21"/>
-      <c r="X21" s="21"/>
-      <c r="Y21" s="21"/>
-    </row>
-    <row r="22" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C22" s="4" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C22" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="23" t="n">
+        <f aca="false">COUNTIF(F9:F16,"Expat")</f>
+        <v>2</v>
+      </c>
+      <c r="E22" s="24" t="s">
         <v>62</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6111,83 +5732,71 @@
         <v>28</v>
       </c>
       <c r="D23" s="23" t="n">
-        <f aca="false">COUNTIF(F9:F17,"Expat")</f>
+        <f aca="false">COUNTIF(F9:F16,"Repatriate")</f>
         <v>3</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C24" s="22" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D24" s="23" t="n">
-        <f aca="false">COUNTIF(F9:F17,"Repatriate")</f>
+        <f aca="false">COUNTIF(F9:F16,"Local")</f>
         <v>3</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="22" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D25" s="23" t="n">
-        <f aca="false">COUNTIF(F9:F17,"Local")</f>
-        <v>3</v>
+        <f aca="false">COUNTIF(H9:H16,"Fixed")</f>
+        <v>7</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C26" s="22" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="D26" s="23" t="n">
-        <f aca="false">COUNTIF(H9:H17,"Fixed")</f>
-        <v>8</v>
+        <f aca="false">COUNTIF(H9:H16,"Rotation")</f>
+        <v>1</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C27" s="22" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="D27" s="23" t="n">
-        <f aca="false">COUNTIF(H9:H17,"Rotation")</f>
-        <v>1</v>
+        <f aca="false">COUNTIF(J9:J16,"Eligible*")</f>
+        <v>3</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="D28" s="23" t="n">
+        <f aca="false">COUNTIF(K9:K16,"Assumption")</f>
+        <v>2</v>
+      </c>
+      <c r="E28" s="24" t="s">
         <v>70</v>
-      </c>
-      <c r="D28" s="23" t="n">
-        <f aca="false">COUNTIF(J9:J17,"Eligible*")</f>
-        <v>3</v>
-      </c>
-      <c r="E28" s="24" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C29" s="22" t="s">
-        <v>72</v>
-      </c>
-      <c r="D29" s="23" t="n">
-        <f aca="false">COUNTIF(K9:K17,"Assumption")</f>
-        <v>2</v>
-      </c>
-      <c r="E29" s="24" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -6195,24 +5804,24 @@
     <mergeCell ref="C3:Y3"/>
     <mergeCell ref="C5:Y5"/>
     <mergeCell ref="C6:Y6"/>
-    <mergeCell ref="C18:L18"/>
-    <mergeCell ref="C21:Y21"/>
+    <mergeCell ref="C17:L17"/>
+    <mergeCell ref="C20:Y20"/>
   </mergeCells>
-  <conditionalFormatting sqref="K9:K17">
+  <conditionalFormatting sqref="K9:K16">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>K9="Assumption"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F9:F17" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F9:F16" type="list">
       <formula1>"Expat,Repatriate,Local"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H9:H17" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H9:H16" type="list">
       <formula1>"Fixed,Rotation"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K9:K17" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K9:K16" type="list">
       <formula1>"Confirmed,Assumption"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6244,7 +5853,7 @@
   <sheetData>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -6259,7 +5868,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -6274,7 +5883,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -6292,147 +5901,147 @@
         <v>6</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="I8" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>81</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C9" s="25" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D9" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="I9" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="J9" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="L9" s="8" t="s">
-        <v>92</v>
-      </c>
       <c r="M9" s="26" t="n">
-        <f aca="false">COUNTIF(Personnel!F9:F17,C9)</f>
-        <v>3</v>
+        <f aca="false">COUNTIF(Personnel!F9:F16,C9)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C10" s="25" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E10" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="I10" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="J10" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="K10" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="L10" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="J10" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>100</v>
-      </c>
       <c r="M10" s="26" t="n">
-        <f aca="false">COUNTIF(Personnel!F9:F17,C10)</f>
+        <f aca="false">COUNTIF(Personnel!F9:F16,C10)</f>
         <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C11" s="25" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E11" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="L11" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="L11" s="8" t="s">
-        <v>104</v>
-      </c>
       <c r="M11" s="26" t="n">
-        <f aca="false">COUNTIF(Personnel!F9:F17,C11)</f>
+        <f aca="false">COUNTIF(Personnel!F9:F16,C11)</f>
         <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C14" s="21" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D14" s="21"/>
       <c r="E14" s="21"/>
@@ -6450,22 +6059,22 @@
         <v>8</v>
       </c>
       <c r="D15" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>106</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>109</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>12</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6473,52 +6082,52 @@
         <v>29</v>
       </c>
       <c r="D16" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="H16" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>113</v>
-      </c>
       <c r="I16" s="26" t="n">
-        <f aca="false">COUNTIF(Personnel!H9:H17,C16)</f>
-        <v>8</v>
+        <f aca="false">COUNTIF(Personnel!H9:H16,C16)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C17" s="25" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D17" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="H17" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="E17" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>117</v>
-      </c>
       <c r="I17" s="26" t="n">
-        <f aca="false">COUNTIF(Personnel!H9:H17,C17)</f>
+        <f aca="false">COUNTIF(Personnel!H9:H16,C17)</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C20" s="27" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D20" s="27"/>
       <c r="E20" s="27"/>

</xml_diff>

<commit_message>
Mark operations support person as TBD
</commit_message>
<xml_diff>
--- a/projects/PetroUrdaneta-FDP9/compensation/personnel_base_salary_contract_types.xlsx
+++ b/projects/PetroUrdaneta-FDP9/compensation/personnel_base_salary_contract_types.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Contract Rules'!$B$2:$M$23</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Personnel!$B$2:$Y$28</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Personnel!$B$2:$Y$30</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -797,40 +797,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Person.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>4</xdr:row>
-                <xdr:rowOff>6</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="F9" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Leticia Almeida has been removed. Operations Support is an open position and the person is to be defined.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -855,7 +822,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F10" authorId="0">
+    <comment ref="F9" authorId="0">
       <text>
         <r>
           <rPr>
@@ -888,7 +855,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F11" authorId="0">
+    <comment ref="F10" authorId="0">
       <text>
         <r>
           <rPr>
@@ -921,7 +888,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F12" authorId="0">
+    <comment ref="F11" authorId="0">
       <text>
         <r>
           <rPr>
@@ -954,7 +921,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F13" authorId="0">
+    <comment ref="F12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -987,7 +954,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F14" authorId="0">
+    <comment ref="F13" authorId="0">
       <text>
         <r>
           <rPr>
@@ -1020,7 +987,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F15" authorId="0">
+    <comment ref="F14" authorId="0">
       <text>
         <r>
           <rPr>
@@ -1053,7 +1020,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="F16" authorId="0">
+    <comment ref="F15" authorId="0">
       <text>
         <r>
           <rPr>
@@ -1086,6 +1053,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="F16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 contract type must be Expat, Repatriate or Local. Edit if management confirms a different classification.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="H9" authorId="0">
       <text>
         <r>
@@ -2117,24 +2117,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Local in Maracaibo or staff house; no cash housing allowance by default.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>16</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Open position. Person, contract type, work arrangement and benefits are to be defined. Salary remains a budget placeholder from the source table.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>21</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -2515,6 +2515,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="C12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default contract rule: TBD</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="C16" authorId="0">
       <text>
         <r>
@@ -2581,6 +2614,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="C18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: TBD</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="C20" authorId="0">
       <text>
         <r>
@@ -2713,15 +2779,15 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D16" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: Continuous assignment to the role</t>
+    <comment ref="D12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default contract rule: Not defined until person and contract are approved</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -2746,15 +2812,15 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="D17" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: Roster-based presence in Venezuela</t>
+    <comment ref="D16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: Continuous assignment to the role</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -2779,6 +2845,72 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="D17" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: Roster-based presence in Venezuela</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: To be determined with the selected Operations Support employee</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="E9" authorId="0">
       <text>
         <r>
@@ -2878,6 +3010,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="E12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. The local payroll and benefit treatment must be reviewed by Venezuelan labor, tax and HR advisers before implementation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>8</xdr:row>
+                <xdr:rowOff>80</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="E16" authorId="0">
       <text>
         <r>
@@ -2944,6 +3109,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="E18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: Not defined</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="F9" authorId="0">
       <text>
         <r>
@@ -3043,6 +3241,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="F12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default contract rule: Not defined</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="F16" authorId="0">
       <text>
         <r>
@@ -3109,6 +3340,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="F18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: Not defined</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="G9" authorId="0">
       <text>
         <r>
@@ -3208,6 +3472,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="G12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default contract rule: Not defined</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="G16" authorId="0">
       <text>
         <r>
@@ -3274,6 +3571,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="G18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: Not defined</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="H9" authorId="0">
       <text>
         <r>
@@ -3373,6 +3703,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="H12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. The local payroll and benefit treatment must be reviewed by Venezuelan labor, tax and HR advisers before implementation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>8</xdr:row>
+                <xdr:rowOff>80</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="H16" authorId="0">
       <text>
         <r>
@@ -3439,6 +3802,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="H18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default work-arrangement rule: Operations Support is an open position.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="I9" authorId="0">
       <text>
         <r>
@@ -3538,7 +3934,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="J9" authorId="0">
+    <comment ref="I12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -3571,7 +3967,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="J10" authorId="0">
+    <comment ref="J9" authorId="0">
       <text>
         <r>
           <rPr>
@@ -3604,7 +4000,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="J11" authorId="0">
+    <comment ref="J10" authorId="0">
       <text>
         <r>
           <rPr>
@@ -3637,6 +4033,72 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="J11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. The local payroll and benefit treatment must be reviewed by Venezuelan labor, tax and HR advisers before implementation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>8</xdr:row>
+                <xdr:rowOff>80</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. The local payroll and benefit treatment must be reviewed by Venezuelan labor, tax and HR advisers before implementation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>8</xdr:row>
+                <xdr:rowOff>80</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="K9" authorId="0">
       <text>
         <r>
@@ -3736,6 +4198,39 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
+    <comment ref="K12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default contract rule: Open position</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
     <comment ref="L9" authorId="0">
       <text>
         <r>
@@ -3828,6 +4323,39 @@
                 <xdr:colOff>55</xdr:colOff>
                 <xdr:row>5</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="L12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default contract rule: Operations Support headcount is budgeted, but the person, contract type and benefits remain to be defined.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -3840,7 +4368,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="128">
   <si>
     <t xml:space="preserve">Personnel — Monthly Base Salary and Contract Classification</t>
   </si>
@@ -4010,7 +4538,13 @@
     <t xml:space="preserve">Operations Support</t>
   </si>
   <si>
-    <t xml:space="preserve">Leticia Almeida</t>
+    <t xml:space="preserve">TBD — Person to be defined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open position. Person, contract type, work arrangement and benefits are to be defined. Salary remains a budget placeholder from the source table.</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL — 8 PEOPLE (COO EXCLUDED)</t>
@@ -4037,12 +4571,24 @@
     <t xml:space="preserve">Local contract from M1 through M12</t>
   </si>
   <si>
+    <t xml:space="preserve">Contract type TBD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open position; contract type is to be defined</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fixed work arrangement</t>
   </si>
   <si>
     <t xml:space="preserve">Rotation work arrangement</t>
   </si>
   <si>
+    <t xml:space="preserve">Work arrangement TBD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open position; work arrangement is to be defined</t>
+  </si>
+  <si>
     <t xml:space="preserve">One-time transition bonuses</t>
   </si>
   <si>
@@ -4058,7 +4604,7 @@
     <t xml:space="preserve">Contract and Benefit Rules by Stage</t>
   </si>
   <si>
-    <t xml:space="preserve">Default policy view — individual packages may override these rules</t>
+    <t xml:space="preserve">Default policy view — individual packages may override these rules | One Operations Support position remains open (TBD)</t>
   </si>
   <si>
     <t xml:space="preserve">M1–M6 is initial stage | From M7 Repatriates operate as Local — Venezuela | Policy is subject to legal and HR validation</t>
@@ -4148,6 +4694,18 @@
     <t xml:space="preserve">No international home leave or expat allowance by default.</t>
   </si>
   <si>
+    <t xml:space="preserve">Not defined until person and contract are approved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not defined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operations Support headcount is budgeted, but the person, contract type and benefits remain to be defined.</t>
+  </si>
+  <si>
     <t xml:space="preserve">WORK ARRANGEMENT RULES</t>
   </si>
   <si>
@@ -4185,6 +4743,12 @@
   </si>
   <si>
     <t xml:space="preserve">Marcelo Dantas is currently shown as Rotation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To be determined with the selected Operations Support employee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operations Support is an open position.</t>
   </si>
   <si>
     <t xml:space="preserve">Policy decision recorded: every Repatriate receives only a one-time M7 transition / repatriation bonus and thereafter is treated as Local — Venezuela. This is not a recurring bonus and is excluded from the monthly base salary. The amount, whether it is salary for Venezuelan labor purposes, the payroll / tax / social-security treatment, immigration status, and local statutory benefits must be approved by Venezuelan legal, tax and HR advisers before implementation. Venezuelan rules apply to employment relationships performed in Venezuela, irrespective of nationality.</t>
@@ -4763,7 +5327,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="C3:Y28"/>
+  <dimension ref="C3:Y30"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="20"/>
@@ -5537,27 +6101,27 @@
         <v>56</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="G16" s="11" t="str">
         <f aca="false">IF(F16="Expat","Yes","No")</f>
         <v>No</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="I16" s="12" t="str">
         <f aca="false">IF(F16="Repatriate","Local — Venezuela",F16)</f>
-        <v>Local</v>
+        <v>TBD</v>
       </c>
       <c r="J16" s="13" t="s">
         <v>41</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="M16" s="15" t="n">
         <f aca="false">$Y16/12</f>
@@ -5613,7 +6177,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C17" s="18" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D17" s="18"/>
       <c r="E17" s="18"/>
@@ -5679,7 +6243,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D20" s="21"/>
       <c r="E20" s="21"/>
@@ -5706,13 +6270,13 @@
     </row>
     <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C21" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5724,7 +6288,7 @@
         <v>2</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5736,7 +6300,7 @@
         <v>3</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5745,58 +6309,82 @@
       </c>
       <c r="D24" s="23" t="n">
         <f aca="false">COUNTIF(F9:F16,"Local")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="22" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="D25" s="23" t="n">
-        <f aca="false">COUNTIF(H9:H16,"Fixed")</f>
-        <v>7</v>
+        <f aca="false">COUNTIF(F9:F16,"TBD")</f>
+        <v>1</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C26" s="22" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="D26" s="23" t="n">
-        <f aca="false">COUNTIF(H9:H16,"Rotation")</f>
-        <v>1</v>
+        <f aca="false">COUNTIF(H9:H16,"Fixed")</f>
+        <v>6</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C27" s="22" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="D27" s="23" t="n">
-        <f aca="false">COUNTIF(J9:J16,"Eligible*")</f>
-        <v>3</v>
+        <f aca="false">COUNTIF(H9:H16,"Rotation")</f>
+        <v>1</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="22" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D28" s="23" t="n">
+        <f aca="false">COUNTIF(H9:H16,"TBD")</f>
+        <v>1</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C29" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="23" t="n">
+        <f aca="false">COUNTIF(J9:J16,"Eligible*")</f>
+        <v>3</v>
+      </c>
+      <c r="E29" s="24" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C30" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="23" t="n">
         <f aca="false">COUNTIF(K9:K16,"Assumption")</f>
-        <v>2</v>
-      </c>
-      <c r="E28" s="24" t="s">
-        <v>70</v>
+        <v>3</v>
+      </c>
+      <c r="E30" s="24" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -5812,13 +6400,23 @@
       <formula>K9="Assumption"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F9:F16">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>F9="TBD"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9:H16">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>H9="TBD"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F9:F16" type="list">
-      <formula1>"Expat,Repatriate,Local"</formula1>
+      <formula1>"Expat,Repatriate,Local,TBD"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H9:H16" type="list">
-      <formula1>"Fixed,Rotation"</formula1>
+      <formula1>"Fixed,Rotation,TBD"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K9:K16" type="list">
@@ -5853,7 +6451,7 @@
   <sheetData>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -5868,7 +6466,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -5883,7 +6481,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="3" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -5901,34 +6499,34 @@
         <v>6</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5936,31 +6534,31 @@
         <v>40</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="J9" s="8" t="s">
         <v>41</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="M9" s="26" t="n">
         <f aca="false">COUNTIF(Personnel!F9:F16,C9)</f>
@@ -5972,31 +6570,31 @@
         <v>28</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="M10" s="26" t="n">
         <f aca="false">COUNTIF(Personnel!F9:F16,C10)</f>
@@ -6008,40 +6606,76 @@
         <v>45</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G11" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="H11" s="8" t="s">
-        <v>93</v>
-      </c>
       <c r="I11" s="8" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="J11" s="8" t="s">
         <v>41</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="M11" s="26" t="n">
         <f aca="false">COUNTIF(Personnel!F9:F16,C11)</f>
-        <v>3</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C12" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="M12" s="26" t="n">
+        <f aca="false">COUNTIF(Personnel!F9:F16,C12)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C14" s="21" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="D14" s="21"/>
       <c r="E14" s="21"/>
@@ -6059,22 +6693,22 @@
         <v>8</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>12</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6082,23 +6716,23 @@
         <v>29</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="I16" s="26" t="n">
         <f aca="false">COUNTIF(Personnel!H9:H16,C16)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6106,28 +6740,52 @@
         <v>50</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="I17" s="26" t="n">
         <f aca="false">COUNTIF(Personnel!H9:H16,C17)</f>
         <v>1</v>
       </c>
     </row>
+    <row r="18" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C18" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="I18" s="26" t="n">
+        <f aca="false">COUNTIF(Personnel!H9:H16,C18)</f>
+        <v>1</v>
+      </c>
+    </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C20" s="27" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="D20" s="27"/>
       <c r="E20" s="27"/>

</xml_diff>

<commit_message>
Add calculated one-time repatriation package
</commit_message>
<xml_diff>
--- a/projects/PetroUrdaneta-FDP9/compensation/personnel_base_salary_contract_types.xlsx
+++ b/projects/PetroUrdaneta-FDP9/compensation/personnel_base_salary_contract_types.xlsx
@@ -9,11 +9,13 @@
   </bookViews>
   <sheets>
     <sheet name="Personnel" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Contract Rules" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Repatriation Package" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Contract Rules" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Contract Rules'!$B$2:$M$23</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'Contract Rules'!$B$2:$M$23</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Personnel!$B$2:$Y$30</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Repatriation Package'!$B$2:$J$38</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -1358,24 +1360,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation package. The core package is currently set at 1.50 months of monthly base salary, with components and caps on the Repatriation Package tab. It does not recur and is excluded from M1–M12 base salary. Payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1391,24 +1393,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation package. The core package is currently set at 1.50 months of monthly base salary, with components and caps on the Repatriation Package tab. It does not recur and is excluded from M1–M12 base salary. Payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1424,24 +1426,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation package. The core package is currently set at 1.50 months of monthly base salary, with components and caps on the Repatriation Package tab. It does not recur and is excluded from M1–M12 base salary. Payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1457,24 +1459,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation package. The core package is currently set at 1.50 months of monthly base salary, with components and caps on the Repatriation Package tab. It does not recur and is excluded from M1–M12 base salary. Payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1490,24 +1492,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation package. The core package is currently set at 1.50 months of monthly base salary, with components and caps on the Repatriation Package tab. It does not recur and is excluded from M1–M12 base salary. Payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1523,24 +1525,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation package. The core package is currently set at 1.50 months of monthly base salary, with components and caps on the Repatriation Package tab. It does not recur and is excluded from M1–M12 base salary. Payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1556,24 +1558,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation package. The core package is currently set at 1.50 months of monthly base salary, with components and caps on the Repatriation Package tab. It does not recur and is excluded from M1–M12 base salary. Payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1589,24 +1591,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation bonus. It does not recur and is excluded from M1–M12 base salary. Amount, payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>9</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. For Repatriates: a single one-time M7 localisation / repatriation package. The core package is currently set at 1.50 months of monthly base salary, with components and caps on the Repatriation Package tab. It does not recur and is excluded from M1–M12 base salary. Payroll treatment and any statutory salary impact require Venezuelan legal, tax and HR confirmation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1886,7 +1888,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; transitions to Local — Venezuela from M7 after the one-time transition package.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -1919,24 +1921,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; initially appointed General Manager of PU on secondment; transitions to Local — Venezuela from M7.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; initially appointed General Manager of PU on secondment; transitions to Local — Venezuela from M7 after the one-time transition package.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>21</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1952,7 +1954,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Repatriate; transitions to Local — Venezuela from M7 after the one-time transition package.</t>
         </r>
       </text>
       <mc:AlternateContent>
@@ -2416,6 +2418,1831 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
+    <comment ref="C10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Core transition package component: Moving &amp; household-goods support</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Core transition package component: Settling-in &amp; incidental expenses</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Core transition package component: Temporary lodging &amp; local setup</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Core transition package component: Local transport &amp; first-mile setup</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Core transition package component: Documentation, payroll &amp; tax onboarding</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C20" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Excluded from one-time package: Base salary</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Excluded from one-time package: Medical insurance</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Excluded from one-time package: Housing / staff house / hotel</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C23" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Excluded from one-time package: Company transport to work</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C24" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Excluded from one-time package: Home leave, stock options, annual incentive and vacation</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C25" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Excluded from one-time package: Venezuelan statutory payroll benefits and taxes</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C30" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Eligible Repatriate identified from Personnel; package is paid once at M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C31" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Eligible Repatriate identified from Personnel; package is paid once at M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C32" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Eligible Repatriate identified from Personnel; package is paid once at M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="C36" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. The package is a company policy item, not a determination of legal or tax treatment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>30</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Editable planning multiplier expressed in months of the employee's monthly base salary.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Editable planning multiplier expressed in months of the employee's monthly base salary.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Editable planning multiplier expressed in months of the employee's monthly base salary.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Editable planning multiplier expressed in months of the employee's monthly base salary.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Editable planning multiplier expressed in months of the employee's monthly base salary.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D20" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Already reflected in M1–M12; not a transition cost.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. M1–M6 and M7+ benefit; not part of the one-time package.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Approved separately by city and individual package; do not duplicate in the allowance.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D23" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Ongoing local benefit, where approved; not a transition payment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D24" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Only where separately approved; not included in the repatriation package.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D25" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Apply according to local legal, tax and payroll review.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D30" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Position.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D31" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Position.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="D32" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: compensation table image pasted_file_yfFQ2v_image.png, provided 7 September 2026; field: Position.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="E10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Paid or reimbursed once at localisation in M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="E11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Paid or reimbursed once at localisation in M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="E12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Paid or reimbursed once at localisation in M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="E13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Paid or reimbursed once at localisation in M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="E14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Paid or reimbursed once at localisation in M7.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Use direct payment or documented reimbursement where practical; do not duplicate other approved benefits.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Use direct payment or documented reimbursement where practical; do not duplicate other approved benefits.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Use direct payment or documented reimbursement where practical; do not duplicate other approved benefits.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Use direct payment or documented reimbursement where practical; do not duplicate other approved benefits.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="F14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Use direct payment or documented reimbursement where practical; do not duplicate other approved benefits.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>6</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="G10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Packing, shipment, excess baggage and local move-related costs.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="G11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Utilities, connection charges, phone / internet setup and small household items.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="G12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Initial hotel or staff-house transition and practical local setup.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="G13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Arrival transport, local mobility and initial work-access setup.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>1</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="G14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Local documentation, payroll onboarding and transition tax consultation.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H10" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. Confirm local payroll, tax and salary-character treatment before payment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>30</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H11" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. Confirm local payroll, tax and salary-character treatment before payment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>30</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. Confirm local payroll, tax and salary-character treatment before payment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>30</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H13" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. Confirm local payroll, tax and salary-character treatment before payment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>30</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="H14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Compliance context: Venezuelan labor rules apply to employment relationships performed in Venezuela regardless of nationality. Source: Embassy of Spain in Caracas, 'Trabajar' (accessed 7 September 2026), summarizing LOTTT. Confirm local payroll, tax and salary-character treatment before payment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>9</xdr:row>
+                <xdr:rowOff>30</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="I30" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Amount, approval and payroll treatment remain subject to Venezuelan legal, tax and HR review.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="I31" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Amount, approval and payroll treatment remain subject to Venezuelan legal, tax and HR review.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="I32" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Amount, approval and payroll treatment remain subject to Venezuelan legal, tax and HR review.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>6</xdr:row>
+                <xdr:rowOff>11</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J30" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. No recurring payment. No housing, medical, statutory benefits or tax gross-up included.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J31" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. No recurring payment. No housing, medical, statutory benefits or tax gross-up included.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+    <comment ref="J32" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. No recurring payment. No housing, medical, statutory benefits or tax gross-up included.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
     <comment ref="C9" authorId="0">
       <text>
         <r>
@@ -4272,24 +6099,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default contract rule: One-time bonus is a transition/localisation support—not an annual incentive. Legal review determines salary and tax treatment.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>79</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>55</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>36</xdr:rowOff>
+          <t xml:space="preserve">Source: management instructions in this task through 7 September 2026. Default contract rule: One-time package covers moving, settling-in, temporary lodging, transport and onboarding support—not an annual incentive. Legal review determines salary and tax treatment.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>55</xdr:colOff>
+                <xdr:row>8</xdr:row>
+                <xdr:rowOff>21</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -4368,7 +6195,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="183">
   <si>
     <t xml:space="preserve">Personnel — Monthly Base Salary and Contract Classification</t>
   </si>
@@ -4460,13 +6287,13 @@
     <t xml:space="preserve">Fixed</t>
   </si>
   <si>
-    <t xml:space="preserve">Eligible — one-time; amount TBD</t>
+    <t xml:space="preserve">Eligible — one-time; 1.50x monthly salary</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed</t>
   </si>
   <si>
-    <t xml:space="preserve">Repatriate; transitions to Local — Venezuela from M7 after the one-time transition bonus.</t>
+    <t xml:space="preserve">Repatriate; transitions to Local — Venezuela from M7 after the one-time transition package.</t>
   </si>
   <si>
     <t xml:space="preserve">Drilling &amp; Well Services Manager</t>
@@ -4475,7 +6302,7 @@
     <t xml:space="preserve">Alexander Stulme</t>
   </si>
   <si>
-    <t xml:space="preserve">Repatriate; initially appointed General Manager of PU on secondment; transitions to Local — Venezuela from M7.</t>
+    <t xml:space="preserve">Repatriate; initially appointed General Manager of PU on secondment; transitions to Local — Venezuela from M7 after the one-time transition package.</t>
   </si>
   <si>
     <t xml:space="preserve">Operations &amp; Maintenance Manager</t>
@@ -4589,10 +6416,10 @@
     <t xml:space="preserve">Open position; work arrangement is to be defined</t>
   </si>
   <si>
-    <t xml:space="preserve">One-time transition bonuses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M7 bonus only; amount is not yet set</t>
+    <t xml:space="preserve">One-time transition packages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7 only; core package = 1.50x monthly salary</t>
   </si>
   <si>
     <t xml:space="preserve">Assumptions to confirm</t>
@@ -4601,6 +6428,171 @@
     <t xml:space="preserve">Editable classifications requiring confirmation</t>
   </si>
   <si>
+    <t xml:space="preserve">One-Time Repatriation / Localisation Transition Package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7 only — moving, settling-in and onboarding costs | Excludes recurring benefits and approved housing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD | Editable assumptions in blue | Multipliers are expressed as months of monthly base salary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORE PACKAGE COMPONENTS — APPLIES ONLY TO REPATRIATES UPON LOCALISATION IN M7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Component</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months of Monthly Salary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Included Costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy Treatment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moving &amp; household-goods support</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time allowance / reimbursement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Packing, shipment, excess baggage and local move-related costs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use documented reimbursement or capped allowance; exclude any recurring storage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Settling-in &amp; incidental expenses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time allowance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilities, connection charges, phone / internet setup and small household items.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capped allowance for incidentals not reimbursed elsewhere.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temporary lodging &amp; local setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time allowance / direct payment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initial hotel or staff-house transition and practical local setup.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use direct company payment where possible; do not duplicate approved housing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local transport &amp; first-mile setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrival transport, local mobility and initial work-access setup.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time transition support; company commuting transport remains a separate local benefit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentation, payroll &amp; tax onboarding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct payment / reimbursement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local documentation, payroll onboarding and transition tax consultation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prefer direct payment or reimbursement against documentation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL CORE PACKAGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXCLUDED FROM THE ONE-TIME PACKAGE — MANAGED SEPARATELY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excluded Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base salary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Already reflected in M1–M12; not a transition cost.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medical insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M1–M6 and M7+ benefit; not part of the one-time package.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Housing / staff house / hotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved separately by city and individual package; do not duplicate in the allowance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company transport to work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ongoing local benefit, where approved; not a transition payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home leave, stock options, annual incentive and vacation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only where separately approved; not included in the repatriation package.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venezuelan statutory payroll benefits and taxes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply according to local legal, tax and payroll review.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7 TRANSITION PACKAGE CALCULATION — REPATRIATES ONLY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly Base Salary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core Package Multiple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-Time Package Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7 Employment Basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approval Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pending individual approval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core 1.50x package; benefits and housing remain outside this calculation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL ONE-TIME M7 PACKAGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy guardrail: the package is a one-time M7 transition support. Use the component-level multipliers above as planning assumptions; pay direct suppliers or reimburse documented costs where possible, and do not duplicate approved housing, hotel, staff-house, medical or transport benefits. Before payment, Venezuelan legal, tax and HR advisers must confirm the correct payroll, tax, social-security and salary-character treatment.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Contract and Benefit Rules by Stage</t>
   </si>
   <si>
@@ -4673,13 +6665,13 @@
     <t xml:space="preserve">Company transport to work; local statutory benefits; any additional benefit requires individual approval</t>
   </si>
   <si>
-    <t xml:space="preserve">Eligible once at M7; amount TBD; not recurring; not in monthly base salary</t>
+    <t xml:space="preserve">Eligible once at M7; core package = 1.50x monthly salary; not recurring; see Repatriation Package</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed policy direction</t>
   </si>
   <si>
-    <t xml:space="preserve">One-time bonus is a transition/localisation support—not an annual incentive. Legal review determines salary and tax treatment.</t>
+    <t xml:space="preserve">One-time package covers moving, settling-in, temporary lodging, transport and onboarding support—not an annual incentive. Legal review determines salary and tax treatment.</t>
   </si>
   <si>
     <t xml:space="preserve">Local — Venezuela</t>
@@ -4751,19 +6743,20 @@
     <t xml:space="preserve">Operations Support is an open position.</t>
   </si>
   <si>
-    <t xml:space="preserve">Policy decision recorded: every Repatriate receives only a one-time M7 transition / repatriation bonus and thereafter is treated as Local — Venezuela. This is not a recurring bonus and is excluded from the monthly base salary. The amount, whether it is salary for Venezuelan labor purposes, the payroll / tax / social-security treatment, immigration status, and local statutory benefits must be approved by Venezuelan legal, tax and HR advisers before implementation. Venezuelan rules apply to employment relationships performed in Venezuela, irrespective of nationality.</t>
+    <t xml:space="preserve">Policy decision recorded: every Repatriate receives only a one-time M7 transition / repatriation package and thereafter is treated as Local — Venezuela. The current core package is 1.50 months of monthly base salary and is itemised on the Repatriation Package tab. It is not a recurring bonus and is excluded from the monthly base salary. The amount, whether it is salary for Venezuelan labor purposes, the payroll / tax / social-security treatment, immigration status, and local statutory benefits must be approved by Venezuelan legal, tax and HR advisers before implementation. Venezuelan rules apply to employment relationships performed in Venezuela, irrespective of nationality.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.0;[RED]&quot;($&quot;#,##0.0\);\-"/>
     <numFmt numFmtId="167" formatCode="#,##0.0;[RED]\(#,##0.0\);\-"/>
     <numFmt numFmtId="168" formatCode="#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.00\x"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -4953,7 +6946,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5058,12 +7051,64 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -6440,6 +8485,468 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="C3:J38"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="36"/>
+  </cols>
+  <sheetData>
+    <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C6" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C8" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
+    </row>
+    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C9" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C10" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="H10" s="27" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C11" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H11" s="27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C12" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" s="26" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="H12" s="27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C13" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="D13" s="26" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="H13" s="27" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C14" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="D14" s="26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="H14" s="27" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C15" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" s="29" t="n">
+        <f aca="false">SUM(D10:D14)</f>
+        <v>1.5</v>
+      </c>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="31"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+    </row>
+    <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C19" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C20" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C21" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="D21" s="27" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C22" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="D22" s="27" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C23" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C24" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="D24" s="27" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C25" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C28" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+    </row>
+    <row r="29" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C29" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C30" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="32" t="n">
+        <f aca="false">VLOOKUP(C30,Personnel!$E$9:$Y$16,21,FALSE())/12</f>
+        <v>18000</v>
+      </c>
+      <c r="F30" s="33" t="n">
+        <f aca="false">$D$15</f>
+        <v>1.5</v>
+      </c>
+      <c r="G30" s="34" t="n">
+        <f aca="false">E30*F30</f>
+        <v>27000</v>
+      </c>
+      <c r="H30" s="35" t="str">
+        <f aca="false">VLOOKUP(C30,Personnel!$E$9:$I$16,5,FALSE())</f>
+        <v>Local — Venezuela</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="J30" s="27" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C31" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E31" s="36" t="n">
+        <f aca="false">VLOOKUP(C31,Personnel!$E$9:$Y$16,21,FALSE())/12</f>
+        <v>15000</v>
+      </c>
+      <c r="F31" s="33" t="n">
+        <f aca="false">$D$15</f>
+        <v>1.5</v>
+      </c>
+      <c r="G31" s="37" t="n">
+        <f aca="false">E31*F31</f>
+        <v>22500</v>
+      </c>
+      <c r="H31" s="35" t="str">
+        <f aca="false">VLOOKUP(C31,Personnel!$E$9:$I$16,5,FALSE())</f>
+        <v>Local — Venezuela</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="J31" s="27" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C32" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" s="36" t="n">
+        <f aca="false">VLOOKUP(C32,Personnel!$E$9:$Y$16,21,FALSE())/12</f>
+        <v>18000</v>
+      </c>
+      <c r="F32" s="33" t="n">
+        <f aca="false">$D$15</f>
+        <v>1.5</v>
+      </c>
+      <c r="G32" s="37" t="n">
+        <f aca="false">E32*F32</f>
+        <v>27000</v>
+      </c>
+      <c r="H32" s="35" t="str">
+        <f aca="false">VLOOKUP(C32,Personnel!$E$9:$I$16,5,FALSE())</f>
+        <v>Local — Venezuela</v>
+      </c>
+      <c r="I32" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="J32" s="27" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C33" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="38" t="n">
+        <f aca="false">SUM(G30:G32)</f>
+        <v>76500</v>
+      </c>
+      <c r="H33" s="30"/>
+      <c r="I33" s="30"/>
+      <c r="J33" s="31"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C36" s="39" t="s">
+        <v>131</v>
+      </c>
+      <c r="D36" s="39"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="39"/>
+      <c r="H36" s="39"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="39"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C37" s="39"/>
+      <c r="D37" s="39"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="39"/>
+      <c r="I37" s="39"/>
+      <c r="J37" s="39"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C38" s="39"/>
+      <c r="D38" s="39"/>
+      <c r="E38" s="39"/>
+      <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
+      <c r="H38" s="39"/>
+      <c r="I38" s="39"/>
+      <c r="J38" s="39"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="C3:J3"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="C28:J28"/>
+    <mergeCell ref="C36:J38"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 Repatriation Package | Page &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="C3:M23"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -6451,7 +8958,7 @@
   <sheetData>
     <row r="3" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C3" s="1" t="s">
-        <v>77</v>
+        <v>132</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -6466,7 +8973,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="2" t="s">
-        <v>78</v>
+        <v>133</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -6481,7 +8988,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="3" t="s">
-        <v>79</v>
+        <v>134</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -6499,34 +9006,34 @@
         <v>6</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>80</v>
+        <v>135</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>81</v>
+        <v>136</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>82</v>
+        <v>137</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>83</v>
+        <v>138</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>84</v>
+        <v>139</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>10</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>85</v>
+        <v>140</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>86</v>
+        <v>141</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>87</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6534,33 +9041,33 @@
         <v>40</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>88</v>
+        <v>143</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>89</v>
+        <v>144</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>92</v>
+        <v>147</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>93</v>
+        <v>148</v>
       </c>
       <c r="J9" s="8" t="s">
         <v>41</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>94</v>
+        <v>149</v>
       </c>
       <c r="L9" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="M9" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="M9" s="40" t="n">
         <f aca="false">COUNTIF(Personnel!F9:F16,C9)</f>
         <v>2</v>
       </c>
@@ -6570,33 +9077,33 @@
         <v>28</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>88</v>
+        <v>143</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>96</v>
+        <v>151</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>97</v>
+        <v>152</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>98</v>
+        <v>153</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>99</v>
+        <v>154</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>102</v>
+        <v>157</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="M10" s="26" t="n">
+        <v>158</v>
+      </c>
+      <c r="M10" s="40" t="n">
         <f aca="false">COUNTIF(Personnel!F9:F16,C10)</f>
         <v>3</v>
       </c>
@@ -6606,33 +9113,33 @@
         <v>45</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>88</v>
+        <v>143</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>104</v>
+        <v>159</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>97</v>
+        <v>152</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>105</v>
+        <v>160</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>99</v>
+        <v>154</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>106</v>
+        <v>161</v>
       </c>
       <c r="J11" s="8" t="s">
         <v>41</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>94</v>
+        <v>149</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="M11" s="26" t="n">
+        <v>162</v>
+      </c>
+      <c r="M11" s="40" t="n">
         <f aca="false">COUNTIF(Personnel!F9:F16,C11)</f>
         <v>2</v>
       </c>
@@ -6642,40 +9149,40 @@
         <v>57</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>108</v>
+        <v>163</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="J12" s="8" t="s">
         <v>41</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>110</v>
+        <v>165</v>
       </c>
       <c r="L12" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="M12" s="26" t="n">
+        <v>166</v>
+      </c>
+      <c r="M12" s="40" t="n">
         <f aca="false">COUNTIF(Personnel!F9:F16,C12)</f>
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C14" s="21" t="s">
-        <v>112</v>
+        <v>167</v>
       </c>
       <c r="D14" s="21"/>
       <c r="E14" s="21"/>
@@ -6693,22 +9200,22 @@
         <v>8</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>113</v>
+        <v>168</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>114</v>
+        <v>169</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>115</v>
+        <v>170</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>116</v>
+        <v>171</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>12</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>87</v>
+        <v>142</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6716,21 +9223,21 @@
         <v>29</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>117</v>
+        <v>172</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>88</v>
+        <v>143</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>118</v>
+        <v>173</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>119</v>
+        <v>174</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I16" s="26" t="n">
+        <v>175</v>
+      </c>
+      <c r="I16" s="40" t="n">
         <f aca="false">COUNTIF(Personnel!H9:H16,C16)</f>
         <v>6</v>
       </c>
@@ -6740,21 +9247,21 @@
         <v>50</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>121</v>
+        <v>176</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>88</v>
+        <v>143</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>122</v>
+        <v>177</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>123</v>
+        <v>178</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="I17" s="26" t="n">
+        <v>179</v>
+      </c>
+      <c r="I17" s="40" t="n">
         <f aca="false">COUNTIF(Personnel!H9:H16,C17)</f>
         <v>1</v>
       </c>
@@ -6764,78 +9271,78 @@
         <v>57</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>125</v>
+        <v>180</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="I18" s="26" t="n">
+        <v>181</v>
+      </c>
+      <c r="I18" s="40" t="n">
         <f aca="false">COUNTIF(Personnel!H9:H16,C18)</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C20" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="27"/>
+      <c r="C20" s="39" t="s">
+        <v>182</v>
+      </c>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="39"/>
+      <c r="I20" s="39"/>
+      <c r="J20" s="39"/>
+      <c r="K20" s="39"/>
+      <c r="L20" s="39"/>
+      <c r="M20" s="39"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="27"/>
-      <c r="K21" s="27"/>
-      <c r="L21" s="27"/>
-      <c r="M21" s="27"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="39"/>
+      <c r="I21" s="39"/>
+      <c r="J21" s="39"/>
+      <c r="K21" s="39"/>
+      <c r="L21" s="39"/>
+      <c r="M21" s="39"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="27"/>
-      <c r="K22" s="27"/>
-      <c r="L22" s="27"/>
-      <c r="M22" s="27"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="39"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="39"/>
+      <c r="I22" s="39"/>
+      <c r="J22" s="39"/>
+      <c r="K22" s="39"/>
+      <c r="L22" s="39"/>
+      <c r="M22" s="39"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="27"/>
-      <c r="M23" s="27"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
+      <c r="K23" s="39"/>
+      <c r="L23" s="39"/>
+      <c r="M23" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>